<commit_message>
v1 of poc done. NEED TO DO: sharepoint addition
</commit_message>
<xml_diff>
--- a/sample_data/comments_sample.xlsx
+++ b/sample_data/comments_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,49 +446,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3a1d6dbd-a81f-4daf-8af9-130983d08791</t>
+          <t>0c6f18e5-1916-4f7d-9059-701de7917f8a</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>This is a great feature request for the dashboard.</t>
+          <t>We need to improve the sync performance for large datasets.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-09T15:46:38.034894</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-09T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0c6f18e5-1916-4f7d-9059-701de7917f8a</t>
+          <t>2da6400c-3da3-42d5-9138-e91eee30ec7a</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>We need to improve the sync performance for large datasets.</t>
+          <t>The user interface is intuitive and easy to use.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-10T15:46:38.034894</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-08-10T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -500,76 +500,76 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2da6400c-3da3-42d5-9138-e91eee30ec7a</t>
+          <t>027b1027-03e8-445e-8667-f6f8c3300913</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The user interface is intuitive and easy to use.</t>
+          <t>Please add more filtering options for the comments.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-11T15:46:38.034894</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-11T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>archived</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>027b1027-03e8-445e-8667-f6f8c3300913</t>
+          <t>771f3157-aa18-4471-ba2d-3b58ba23a3e3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Please add more filtering options for the comments.</t>
+          <t>Consider adding export functionality to Excel.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-12T15:46:38.034894</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-12T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>771f3157-aa18-4471-ba2d-3b58ba23a3e3</t>
+          <t>e7550e16-a6c5-4a24-b427-cca4001053d1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Consider adding export functionality to Excel.</t>
+          <t>The two-way sync is working perfectly.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-13T15:46:38.034894</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-13T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -581,76 +581,76 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>e7550e16-a6c5-4a24-b427-cca4001053d1</t>
+          <t>01161e1e-438b-4d7f-bdc0-4c99e7c5da9b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>The two-way sync is working perfectly.</t>
+          <t>We should implement conflict resolution in future versions.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-14T15:46:38.034894</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-14T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>archived</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>01161e1e-438b-4d7f-bdc0-4c99e7c5da9b</t>
+          <t>3caa99d0-a329-48e8-8a39-079d88fd2686</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>We should implement conflict resolution in future versions.</t>
+          <t>The API integration with Smartsheets is seamless.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-15T15:46:38.034894</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-15T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>archived</t>
+          <t>active</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3caa99d0-a329-48e8-8a39-079d88fd2686</t>
+          <t>81799047-aec2-4e4b-beb7-37a7761106b0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>The API integration with Smartsheets is seamless.</t>
+          <t>Add support for bulk operations in the next release.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-16T15:46:38.034894</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-16T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -662,54 +662,189 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>81799047-aec2-4e4b-beb7-37a7761106b0</t>
+          <t>5bd26001-5efd-4d39-8ab1-28c5985d7688</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Add support for bulk operations in the next release.</t>
+          <t>Documentation is clear and helpful for setup.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-17T15:46:38.034894</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-17T17:46:38.034894</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>archived</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5bd26001-5efd-4d39-8ab1-28c5985d7688</t>
+          <t>043fa6f5-3ce5-4410-9263-57032bfeb496</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Documentation is clear and helpful for setup.</t>
+          <t>Testing this from Kush interactive dashboard</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-18T15:46:38.034894</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-18T17:46:38.034894</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>17a850b9-091e-46f2-90dd-bc4747f1d172</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>testing ui improvement</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3a1d6dbd-a81f-4daf-8af9-130983d08791</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>This is a great feature request for the dashboard.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>archived</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>01161e1e-438b-4d7f-bdc0-4c99e7c5da9d</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>I am adding this manually in excel</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>69265f0d-3a5e-4d08-8cf6-759ee94a2c1c</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>yoo will u appear in exceL?</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>69265f0d-3a5e-4d08-8cf6-759ee94a2c1c</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>yoo will u appear in exceL?</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
made grid changes + added columns + age of
</commit_message>
<xml_diff>
--- a/sample_data/comments_sample.xlsx
+++ b/sample_data/comments_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,429 +424,881 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>comment_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>comment_text</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>aging_bucket</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>start_date</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>account</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pl_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>sub_program</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>created_date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>modified_date</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>status</t>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>paired_comment_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>flag_reason</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>flagged_date</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0c6f18e5-1916-4f7d-9059-701de7917f8a</t>
+          <t>51528ab7-360f-4caa-add0-24c0582954c8</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>We need to improve the sync performance for large datasets.</t>
+          <t>Northwind Renewal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>This is a great feature request for the dashboard.</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>ACCT-1000</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>P&amp;L A</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SP-0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2da6400c-3da3-42d5-9138-e91eee30ec7a</t>
+          <t>55d807ef-b735-4683-89c8-2e92db7ddddf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>The user interface is intuitive and easy to use.</t>
+          <t>Contoso Invoice</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>We need to improve the sync performance for large datasets.</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ACCT-1001</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>P&amp;L B</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SP-1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>027b1027-03e8-445e-8667-f6f8c3300913</t>
+          <t>a90ea6f1-fc13-4bdd-a0e0-64ec75d843e2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Please add more filtering options for the comments.</t>
+          <t>Fabrikam Follow-up</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>The user interface is intuitive and easy to use.</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>30</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>archived</t>
-        </is>
-      </c>
+          <t>0-30</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>ACCT-1002</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>P&amp;L C</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SP-2</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>771f3157-aa18-4471-ba2d-3b58ba23a3e3</t>
+          <t>c068b4a0-bc81-4121-b682-6f163ae001bb</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Consider adding export functionality to Excel.</t>
+          <t>Adventure Works</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>Please add more filtering options for the comments.</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>31</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>31-60</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ACCT-1003</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>P&amp;L D</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SP-3</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>e7550e16-a6c5-4a24-b427-cca4001053d1</t>
+          <t>ebaf69ea-cb14-475d-8a9e-49411473e969</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>The two-way sync is working perfectly.</t>
+          <t>Tailspin Payment</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>Consider adding export functionality to Excel.</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>60</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>31-60</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ACCT-1004</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>P&amp;L A</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>SP-4</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01161e1e-438b-4d7f-bdc0-4c99e7c5da9b</t>
+          <t>8317bc9b-16da-4250-91fb-249aa6acfc28</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>We should implement conflict resolution in future versions.</t>
+          <t>Woodgrove Account</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>The two-way sync is working perfectly.</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>61</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>archived</t>
-        </is>
-      </c>
+          <t>61-90</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>ACCT-1005</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>P&amp;L B</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>SP-0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3caa99d0-a329-48e8-8a39-079d88fd2686</t>
+          <t>f35c418e-cdc1-4ed1-ad82-fd449258afaf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>The API integration with Smartsheets is seamless.</t>
+          <t>Litware Review</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>We should implement conflict resolution in future versions.</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>90</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>61-90</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>ACCT-1006</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>P&amp;L C</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>SP-1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>81799047-aec2-4e4b-beb7-37a7761106b0</t>
+          <t>8e011c47-29eb-4dad-9eee-9d0e710c97bd</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Add support for bulk operations in the next release.</t>
+          <t>Proseware Balance</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>The API integration with Smartsheets is seamless.</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>120</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>91-180</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>ACCT-1007</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>P&amp;L D</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SP-2</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5bd26001-5efd-4d39-8ab1-28c5985d7688</t>
+          <t>4dcf51cf-1eb7-424a-9dca-2abe9f6a2c00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Documentation is clear and helpful for setup.</t>
+          <t>Alpine Ski House</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>Add support for bulk operations in the next release.</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>180</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>archived</t>
-        </is>
-      </c>
+          <t>91-180</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-04-08</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>ACCT-1008</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>P&amp;L A</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>SP-3</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>043fa6f5-3ce5-4410-9263-57032bfeb496</t>
+          <t>ffca5283-84fa-4339-a5bc-a41fae41b283</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Testing this from Kush interactive dashboard</t>
+          <t>Blue Yonder</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
+          <t>Documentation is clear and helpful for setup.</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>240</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>180+</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>ACCT-1009</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>P&amp;L B</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>SP-4</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17a850b9-091e-46f2-90dd-bc4747f1d172</t>
+          <t>ae32641d-7f1a-404e-9a49-ea3091474adb</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>testing ui improvement</t>
+          <t>Wide World Importers</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
+          <t>Payment details need leadership review.</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>365</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>180+</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2025-10-05</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>ACCT-1010</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>P&amp;L C</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>SP-0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>3a1d6dbd-a81f-4daf-8af9-130983d08791</t>
+          <t>e3aca988-d424-49f1-a98f-0e37b045ccc8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>This is a great feature request for the dashboard.</t>
+          <t>Consolidated Messenger</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>Account has reached the escalation threshold.</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>500</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>archived</t>
-        </is>
-      </c>
+          <t>180+</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2025-05-23</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>ACCT-1011</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>P&amp;L D</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>SP-1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>01161e1e-438b-4d7f-bdc0-4c99e7c5da9d</t>
+          <t>8c1420d9-ea54-414a-950d-2b59a99fbd06</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>I am adding this manually in excel</t>
+          <t>Humongous Insurance</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>Account is beyond the escalation threshold.</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>501</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>180+</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025-05-22</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ACCT-1012</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>P&amp;L A</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>SP-2</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>69265f0d-3a5e-4d08-8cf6-759ee94a2c1c</t>
+          <t>e265b118-b670-46a9-ae28-b8426fdefa3a</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>yoo will u appear in exceL?</t>
+          <t>Lucerne Publishing</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
+          <t>Long-running balance requires immediate action.</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>540</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>active</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>69265f0d-3a5e-4d08-8cf6-759ee94a2c1c</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>yoo will u appear in exceL?</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
+          <t>180+</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2025-04-13</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>ACCT-1013</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>P&amp;L B</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>SP-3</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>